<commit_message>
Dataset update: removing reverters that were in MCI/AD group due to bug in detect_reverters funciton.
</commit_message>
<xml_diff>
--- a/group_visit_counts.xlsx
+++ b/group_visit_counts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aeg00011/Desktop/AD-Research/AD-Early-Prediction/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D830531-5600-6C4D-A737-8B6B75B1BE0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25F246C3-A5AE-394C-B199-31DB448653D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-35220" yWindow="940" windowWidth="30240" windowHeight="17260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -462,7 +462,7 @@
         <v>353</v>
       </c>
       <c r="E3" s="1">
-        <v>317</v>
+        <v>310</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -479,7 +479,7 @@
         <v>174</v>
       </c>
       <c r="E4" s="1">
-        <v>280</v>
+        <v>268</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -496,7 +496,7 @@
         <v>81</v>
       </c>
       <c r="E5" s="1">
-        <v>185</v>
+        <v>176</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -513,7 +513,7 @@
         <v>59</v>
       </c>
       <c r="E6" s="1">
-        <v>138</v>
+        <v>132</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -530,7 +530,7 @@
         <v>41</v>
       </c>
       <c r="E7" s="1">
-        <v>127</v>
+        <v>118</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -547,7 +547,7 @@
         <v>20</v>
       </c>
       <c r="E8" s="1">
-        <v>83</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -564,7 +564,7 @@
         <v>9</v>
       </c>
       <c r="E9" s="1">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
@@ -581,7 +581,7 @@
         <v>11</v>
       </c>
       <c r="E10" s="1">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>